<commit_message>
feat: add audit result for 2025-07-08
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+  <si>
+    <t>wga.hu</t>
+  </si>
   <si>
     <t>freeweb.hu</t>
   </si>
@@ -374,6 +377,12 @@
   </si>
   <si>
     <t>pirateclub.hu</t>
+  </si>
+  <si>
+    <t>handbook.hu</t>
+  </si>
+  <si>
+    <t>travelo.hu</t>
   </si>
 </sst>
 </file>
@@ -750,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A121"/>
+  <dimension ref="A1:A124"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1358,6 +1367,21 @@
         <v>120</v>
       </c>
     </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: update list of failed domains
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t>wga.hu</t>
   </si>
@@ -383,6 +383,9 @@
   </si>
   <si>
     <t>travelo.hu</t>
+  </si>
+  <si>
+    <t>lebelier.hu</t>
   </si>
 </sst>
 </file>
@@ -759,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A124"/>
+  <dimension ref="A1:A125"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1382,6 +1385,11 @@
         <v>123</v>
       </c>
     </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>124</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-07-22
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
   <si>
     <t>wga.hu</t>
   </si>
@@ -386,6 +386,15 @@
   </si>
   <si>
     <t>lebelier.hu</t>
+  </si>
+  <si>
+    <t>m4sportelo.hu</t>
+  </si>
+  <si>
+    <t>zoldlepes.hu</t>
+  </si>
+  <si>
+    <t>kreativ.hu</t>
   </si>
 </sst>
 </file>
@@ -762,7 +771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A125"/>
+  <dimension ref="A1:A128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1390,6 +1399,21 @@
         <v>124</v>
       </c>
     </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-07-29
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t>wga.hu</t>
   </si>
@@ -395,6 +395,9 @@
   </si>
   <si>
     <t>kreativ.hu</t>
+  </si>
+  <si>
+    <t>lovasok.hu</t>
   </si>
 </sst>
 </file>
@@ -771,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A128"/>
+  <dimension ref="A1:A129"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1414,6 +1417,11 @@
         <v>127</v>
       </c>
     </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>128</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-08-05
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -1,12 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10727"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE583F4C-0C48-4C4C-9C38-173DEAC80EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="failed_domains" state="visible" r:id="rId4"/>
+    <sheet name="failed_domains" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -403,14 +420,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -773,657 +790,657 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A129"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>128</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add audit result for 2025-08-12
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -1,34 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10727"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE583F4C-0C48-4C4C-9C38-173DEAC80EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="failed_domains" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="failed_domains" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
   <si>
     <t>wga.hu</t>
   </si>
@@ -415,19 +398,37 @@
   </si>
   <si>
     <t>lovasok.hu</t>
+  </si>
+  <si>
+    <t>greenaqua.hu</t>
+  </si>
+  <si>
+    <t>gazdabolt.hu</t>
+  </si>
+  <si>
+    <t>okosdoboz.hu</t>
+  </si>
+  <si>
+    <t>polomania.hu</t>
+  </si>
+  <si>
+    <t>molfehervarfc.hu</t>
+  </si>
+  <si>
+    <t>kozelben.hu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -790,657 +791,687 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A129"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A135"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>128</v>
       </c>
     </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add audit result for 2025-08-19
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>wga.hu</t>
   </si>
@@ -416,6 +416,12 @@
   </si>
   <si>
     <t>kozelben.hu</t>
+  </si>
+  <si>
+    <t>meduzaingatlan.hu</t>
+  </si>
+  <si>
+    <t>bpbutor.hu</t>
   </si>
 </sst>
 </file>
@@ -792,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A135"/>
+  <dimension ref="A1:A137"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1470,6 +1476,16 @@
         <v>134</v>
       </c>
     </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>136</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-08-26
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
   <si>
     <t>wga.hu</t>
   </si>
@@ -422,6 +422,9 @@
   </si>
   <si>
     <t>bpbutor.hu</t>
+  </si>
+  <si>
+    <t>kormanyhivatal.hu</t>
   </si>
 </sst>
 </file>
@@ -798,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A137"/>
+  <dimension ref="A1:A138"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1486,6 +1489,11 @@
         <v>136</v>
       </c>
     </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-09-02
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t>wga.hu</t>
   </si>
@@ -425,6 +425,9 @@
   </si>
   <si>
     <t>kormanyhivatal.hu</t>
+  </si>
+  <si>
+    <t>deninet.hu</t>
   </si>
 </sst>
 </file>
@@ -801,7 +804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A138"/>
+  <dimension ref="A1:A139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1494,6 +1497,11 @@
         <v>137</v>
       </c>
     </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>138</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-09-09
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>wga.hu</t>
   </si>
@@ -428,6 +428,9 @@
   </si>
   <si>
     <t>deninet.hu</t>
+  </si>
+  <si>
+    <t>egy.hu</t>
   </si>
 </sst>
 </file>
@@ -804,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A139"/>
+  <dimension ref="A1:A140"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1502,6 +1505,11 @@
         <v>138</v>
       </c>
     </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>139</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-09-16
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t>wga.hu</t>
   </si>
@@ -431,6 +431,12 @@
   </si>
   <si>
     <t>egy.hu</t>
+  </si>
+  <si>
+    <t>agraroldal.hu</t>
+  </si>
+  <si>
+    <t>jatekbolt.hu</t>
   </si>
 </sst>
 </file>
@@ -807,7 +813,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A140"/>
+  <dimension ref="A1:A142"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1510,6 +1516,16 @@
         <v>139</v>
       </c>
     </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>141</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-09-23
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
   <si>
     <t>wga.hu</t>
   </si>
@@ -437,6 +437,12 @@
   </si>
   <si>
     <t>jatekbolt.hu</t>
+  </si>
+  <si>
+    <t>pingvinpatika.hu</t>
+  </si>
+  <si>
+    <t>termalonline.hu</t>
   </si>
 </sst>
 </file>
@@ -813,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A142"/>
+  <dimension ref="A1:A144"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1526,6 +1532,16 @@
         <v>141</v>
       </c>
     </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>143</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-09-30
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t>wga.hu</t>
   </si>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t>termalonline.hu</t>
+  </si>
+  <si>
+    <t>laptophardware.hu</t>
   </si>
 </sst>
 </file>
@@ -819,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A144"/>
+  <dimension ref="A1:A145"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1542,6 +1545,11 @@
         <v>143</v>
       </c>
     </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>144</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-10-14
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
   <si>
     <t>wga.hu</t>
   </si>
@@ -446,6 +446,9 @@
   </si>
   <si>
     <t>laptophardware.hu</t>
+  </si>
+  <si>
+    <t>met.hu</t>
   </si>
 </sst>
 </file>
@@ -822,7 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A145"/>
+  <dimension ref="A1:A146"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1550,6 +1553,11 @@
         <v>144</v>
       </c>
     </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>145</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-10-21
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t>wga.hu</t>
   </si>
@@ -449,6 +449,9 @@
   </si>
   <si>
     <t>met.hu</t>
+  </si>
+  <si>
+    <t>studyinhungary.hu</t>
   </si>
 </sst>
 </file>
@@ -825,7 +828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A146"/>
+  <dimension ref="A1:A147"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1558,6 +1561,11 @@
         <v>145</v>
       </c>
     </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>146</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-11-04
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>wga.hu</t>
   </si>
@@ -452,6 +452,12 @@
   </si>
   <si>
     <t>studyinhungary.hu</t>
+  </si>
+  <si>
+    <t>jatekneked.hu</t>
+  </si>
+  <si>
+    <t>laskod.hu</t>
   </si>
 </sst>
 </file>
@@ -828,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A147"/>
+  <dimension ref="A1:A149"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1566,6 +1572,16 @@
         <v>146</v>
       </c>
     </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>148</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-11-11
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="151">
   <si>
     <t>wga.hu</t>
   </si>
@@ -458,6 +458,12 @@
   </si>
   <si>
     <t>laskod.hu</t>
+  </si>
+  <si>
+    <t>mellrakforum.hu</t>
+  </si>
+  <si>
+    <t>alternativenergia.hu</t>
   </si>
 </sst>
 </file>
@@ -834,7 +840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A149"/>
+  <dimension ref="A1:A151"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1582,6 +1588,16 @@
         <v>148</v>
       </c>
     </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-11-18
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t>wga.hu</t>
   </si>
@@ -464,6 +464,12 @@
   </si>
   <si>
     <t>alternativenergia.hu</t>
+  </si>
+  <si>
+    <t>valtanek.hu</t>
+  </si>
+  <si>
+    <t>neprajz.hu</t>
   </si>
 </sst>
 </file>
@@ -840,7 +846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A151"/>
+  <dimension ref="A1:A153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1598,6 +1604,16 @@
         <v>150</v>
       </c>
     </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-11-25
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
   <si>
     <t>wga.hu</t>
   </si>
@@ -470,6 +470,12 @@
   </si>
   <si>
     <t>neprajz.hu</t>
+  </si>
+  <si>
+    <t>news7.hu</t>
+  </si>
+  <si>
+    <t>eblog.hu</t>
   </si>
 </sst>
 </file>
@@ -846,7 +852,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A153"/>
+  <dimension ref="A1:A155"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1614,6 +1620,16 @@
         <v>152</v>
       </c>
     </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>154</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-12-02
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
     <t>wga.hu</t>
   </si>
@@ -476,6 +476,9 @@
   </si>
   <si>
     <t>eblog.hu</t>
+  </si>
+  <si>
+    <t>ventil.hu</t>
   </si>
 </sst>
 </file>
@@ -852,7 +855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A155"/>
+  <dimension ref="A1:A156"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1630,6 +1633,11 @@
         <v>154</v>
       </c>
     </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>155</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-12-16
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
   <si>
     <t>wga.hu</t>
   </si>
@@ -479,6 +479,9 @@
   </si>
   <si>
     <t>ventil.hu</t>
+  </si>
+  <si>
+    <t>rtlplusz.hu</t>
   </si>
 </sst>
 </file>
@@ -855,7 +858,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A156"/>
+  <dimension ref="A1:A157"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1638,6 +1641,11 @@
         <v>155</v>
       </c>
     </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat: add audit result for 2025-12-23
</commit_message>
<xml_diff>
--- a/data/processed/failed_domains.xlsx
+++ b/data/processed/failed_domains.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t>wga.hu</t>
   </si>
@@ -482,6 +482,9 @@
   </si>
   <si>
     <t>rtlplusz.hu</t>
+  </si>
+  <si>
+    <t>keptelenseg.hu</t>
   </si>
 </sst>
 </file>
@@ -858,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A157"/>
+  <dimension ref="A1:A158"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1646,6 +1649,11 @@
         <v>156</v>
       </c>
     </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>